<commit_message>
feat(F00): harden app connections
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5576,9 +5576,9 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="J2" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="J2" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="20" t="inlineStr">
@@ -5591,14 +5591,14 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="M2" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N2" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="M2" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N2" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O2" s="20" t="inlineStr">
@@ -5607,11 +5607,11 @@
         </is>
       </c>
       <c r="P2" s="21" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="Q2" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R2" s="18" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="T2" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>local-g4-security</t>
         </is>
       </c>
       <c r="U2" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V2" s="18" t="inlineStr">
         <is>
-          <t>2026-07-16T22:31:50.345Z</t>
+          <t>2026-07-17T07:56:12.726Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F00): finalize integration tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5601,13 +5601,13 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O2" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O2" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P2" s="21" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="Q2" s="18" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="U2" s="18" t="inlineStr">
         <is>
-          <t>In-Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V2" s="18" t="inlineStr">

</xml_diff>

<commit_message>
chore: claim parallel Wave 1 builders
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5656,9 +5656,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -5717,11 +5717,11 @@
         </is>
       </c>
       <c r="P3" s="21" t="n">
-        <v>0</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="Q3" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="R3" s="18" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="S3" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f01-builder</t>
         </is>
       </c>
       <c r="T3" s="18" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="V3" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T08:08:10.803Z</t>
         </is>
       </c>
     </row>
@@ -5876,9 +5876,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -5937,11 +5937,11 @@
         </is>
       </c>
       <c r="P5" s="21" t="n">
-        <v>0</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="Q5" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="R5" s="18" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="S5" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f03-builder</t>
         </is>
       </c>
       <c r="T5" s="18" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="V5" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T08:08:17.364Z</t>
         </is>
       </c>
     </row>
@@ -6096,9 +6096,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -6157,11 +6157,11 @@
         </is>
       </c>
       <c r="P7" s="21" t="n">
-        <v>0</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="R7" s="18" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="S7" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f05-builder</t>
         </is>
       </c>
       <c r="T7" s="18" t="inlineStr">
@@ -6186,7 +6186,7 @@
       </c>
       <c r="V7" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T08:08:24.742Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: claim F14 metrics builder
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7086,9 +7086,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
@@ -7147,11 +7147,11 @@
         </is>
       </c>
       <c r="P16" s="21" t="n">
-        <v>0</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="Q16" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="R16" s="18" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="S16" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f14-builder</t>
         </is>
       </c>
       <c r="T16" s="18" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="V16" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T08:20:16.662Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: claim F22 discovery builder
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7966,9 +7966,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
@@ -8027,11 +8027,11 @@
         </is>
       </c>
       <c r="P24" s="21" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Q24" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="R24" s="18" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="S24" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f22-builder</t>
         </is>
       </c>
       <c r="T24" s="18" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="V24" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T08:22:03.702Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F05): mark integration complete
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6101,67 +6101,67 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O7" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O7" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P7" s="21" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R7" s="18" t="inlineStr">
@@ -6181,12 +6181,12 @@
       </c>
       <c r="U7" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V7" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:08:24.742Z</t>
+          <t>2026-07-17T08:39:09.741Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F03): mark integration handoff complete
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5881,67 +5881,67 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O5" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O5" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P5" s="21" t="n">
-        <v>0.08333333333333333</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R5" s="18" t="inlineStr">
@@ -5961,12 +5961,12 @@
       </c>
       <c r="U5" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Ready-for-integration</t>
         </is>
       </c>
       <c r="V5" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:08:17.364Z</t>
+          <t>2026-07-17T08:52:21.659Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F01): mark schema contracts complete
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5661,67 +5661,67 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O3" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O3" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P3" s="21" t="n">
-        <v>0.08333333333333333</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G8</t>
         </is>
       </c>
       <c r="R3" s="18" t="inlineStr">
@@ -5741,12 +5741,12 @@
       </c>
       <c r="U3" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V3" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:08:10.803Z</t>
+          <t>2026-07-17T09:12:37.704Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(F14): preserve stats response envelope
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7091,67 +7091,67 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N16" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K16" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N16" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O16" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O16" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P16" s="21" t="n">
-        <v>0.1111111111111111</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G8</t>
         </is>
       </c>
       <c r="R16" s="18" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="U16" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V16" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:20:16.662Z</t>
+          <t>2026-07-17T09:22:44.597Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F19): record completion status
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7636,72 +7636,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O21" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O21" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P21" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R21" s="18" t="inlineStr">
@@ -7721,12 +7721,12 @@
       </c>
       <c r="U21" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Ready-for-integration</t>
         </is>
       </c>
       <c r="V21" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T09:44:53.321Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: checkpoint Wave 1 tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5961,12 +5961,12 @@
       </c>
       <c r="U5" s="18" t="inlineStr">
         <is>
-          <t>Ready-for-integration</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V5" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:52:21.659Z</t>
+          <t>2026-07-17T09:48:38.792Z</t>
         </is>
       </c>
     </row>
@@ -6181,12 +6181,12 @@
       </c>
       <c r="U7" s="18" t="inlineStr">
         <is>
-          <t>In-Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V7" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:39:09.741Z</t>
+          <t>2026-07-17T09:48:38.865Z</t>
         </is>
       </c>
     </row>
@@ -7721,12 +7721,12 @@
       </c>
       <c r="U21" s="18" t="inlineStr">
         <is>
-          <t>Ready-for-integration</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V21" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T09:44:53.321Z</t>
+          <t>2026-07-17T09:48:38.943Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add F02 drift detection
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5766,72 +5766,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O4" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P4" s="21" t="n">
-        <v>0</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G8</t>
         </is>
       </c>
       <c r="R4" s="18" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="S4" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>f02-builder</t>
         </is>
       </c>
       <c r="T4" s="18" t="inlineStr">
@@ -5851,12 +5851,12 @@
       </c>
       <c r="U4" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V4" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T10:03:55.472Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: finalize F02 integration tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5831,7 +5831,7 @@
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
-          <t>G8</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R4" s="18" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="V4" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T10:17:30.790Z</t>
+          <t>2026-07-17T10:24:43.808Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: finalize F10 integration tracking
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6646,14 +6646,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
@@ -6661,24 +6661,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K12" s="22" t="inlineStr">
@@ -6686,14 +6686,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="L12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="N12" s="22" t="inlineStr">
@@ -6701,17 +6701,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O12" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O12" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P12" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R12" s="18" t="inlineStr">
@@ -6731,12 +6731,12 @@
       </c>
       <c r="U12" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V12" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T10:31:26.160Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F16): finalize integration tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7306,14 +7306,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -7321,57 +7321,57 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="G18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K18" s="22" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N18" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N18" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O18" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O18" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P18" s="21" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="Q18" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R18" s="18" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="S18" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>feat/F16-result-cache</t>
         </is>
       </c>
       <c r="T18" s="18" t="inlineStr">
@@ -7391,12 +7391,12 @@
       </c>
       <c r="U18" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V18" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T11:03:33.628Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F23): finalize integration tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -8076,72 +8076,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I25" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O25" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O25" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P25" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R25" s="18" t="inlineStr">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="S25" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex</t>
         </is>
       </c>
       <c r="T25" s="18" t="inlineStr">
@@ -8161,12 +8161,12 @@
       </c>
       <c r="U25" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V25" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T11:10:29.082Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F22): finalize integration tracker
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -7971,34 +7971,34 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K24" s="22" t="inlineStr">
@@ -8006,14 +8006,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="L24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="L24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="N24" s="22" t="inlineStr">
@@ -8021,17 +8021,17 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O24" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O24" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P24" s="21" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Q24" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R24" s="18" t="inlineStr">
@@ -8051,12 +8051,12 @@
       </c>
       <c r="U24" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V24" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T08:22:03.702Z</t>
+          <t>2026-07-17T11:22:39.595Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(engine): add CEL conditional branching
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6426,14 +6426,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr">
@@ -6441,57 +6441,57 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P10" s="21" t="n">
-        <v>0</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="Q10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R10" s="18" t="inlineStr">
@@ -6511,12 +6511,12 @@
       </c>
       <c r="U10" s="18" t="inlineStr">
         <is>
-          <t>In-Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V10" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T12:01:46.568Z</t>
+          <t>2026-07-17T12:18:17.690Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add template pipelines
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6316,72 +6316,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P9" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G8</t>
         </is>
       </c>
       <c r="R9" s="18" t="inlineStr">
@@ -6401,12 +6401,12 @@
       </c>
       <c r="U9" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V9" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T12:14:48.489Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add self-healing template workflow
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5986,59 +5986,59 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="O6" s="20" t="inlineStr">
@@ -6047,11 +6047,11 @@
         </is>
       </c>
       <c r="P6" s="21" t="n">
-        <v>0</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R6" s="18" t="inlineStr">
@@ -6061,22 +6061,22 @@
       </c>
       <c r="S6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex</t>
         </is>
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex-self-review</t>
         </is>
       </c>
       <c r="U6" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T12:24:34.685Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(F04): normalize registry repo path and redact PR dry-run output
Addresses gate findings: registry-client.ts now resolves
APIMEMCP_REGISTRY_REPO_PATH (including Windows drive paths) to a
file:// URL before git clone instead of passing a raw local path.
self-heal.ts no longer serializes full dry-run output into the PR
body; it emits a redacted type/size/key summary instead.

Build and full test suite (108 tests) pass locally. Tracker left at
G1/In-Review pending independent gate review, not marked Done.
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -135,7 +135,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00FCD34D"/>
       </patternFill>
     </fill>
     <fill>
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -239,11 +239,12 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5978,12 +5979,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>F04</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Self-healing templates</t>
         </is>
@@ -6048,9 +6049,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O6" s="23" t="inlineStr">
+        <is>
+          <t>In-Review</t>
         </is>
       </c>
       <c r="P6" s="21" t="n">
@@ -6058,12 +6059,12 @@
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R6" s="18" t="inlineStr">
         <is>
-          <t>G1 npm test fails in openTemplatePr local git clone on Windows; G6 verify-F04 fails at same local registry clone path; G4 review also finds PR body includes full dry-run output.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S6" s="18" t="inlineStr">
@@ -6078,12 +6079,12 @@
       </c>
       <c r="U6" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V6" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T12:47:05.174Z</t>
+          <t>2026-07-17T13:04:41.588Z</t>
         </is>
       </c>
     </row>
@@ -11268,9 +11269,9 @@
       <c r="L6" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="M6" s="27" t="inlineStr">
-        <is>
-          <t>Late</t>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>On-track</t>
         </is>
       </c>
       <c r="N6" s="24" t="inlineStr">

</xml_diff>

<commit_message>
chore: regenerate tracker workbook post F07/F08 merge, update orchestration log
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5827,7 +5827,7 @@
         </is>
       </c>
       <c r="P4" s="21" t="n">
-        <v>0.9090909090909091</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
@@ -6157,7 +6157,7 @@
         </is>
       </c>
       <c r="P7" s="21" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
@@ -6426,14 +6426,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr">
@@ -6441,57 +6441,57 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P10" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R10" s="18" t="inlineStr">
@@ -6506,17 +6506,17 @@
       </c>
       <c r="T10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Codex_F08_gate_reviewer</t>
         </is>
       </c>
       <c r="U10" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T12:52:18.246Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F12): implement policy engine for extraction rules
- Add src/policy.ts: enforcePolicy function with rate limiting, robots.txt compliance, and ToS domain restrictions
- Modify engine.ts: call enforcePolicy before page navigation with template ID and target URL
- Update extraction-runner.ts: pass templateId through to executeExtraction
- Add comprehensive unit tests in src/policy.test.ts covering rate limiting, robots.txt parsing, ToS blocking, and error handling
- Add verify-F12.mjs script for live verification with local fixture server
- All tests green; build clean
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6031,9 +6031,9 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="M6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="M6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="N6" s="20" t="inlineStr">
@@ -6047,11 +6047,11 @@
         </is>
       </c>
       <c r="P6" s="21" t="n">
-        <v>0</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="R6" s="18" t="inlineStr">
@@ -6066,17 +6066,17 @@
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex-f04-g2-reviewer</t>
         </is>
       </c>
       <c r="U6" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T13:53:48.545Z</t>
         </is>
       </c>
     </row>
@@ -6786,9 +6786,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K13" s="22" t="inlineStr">
@@ -6801,9 +6801,9 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="M13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="M13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="N13" s="22" t="inlineStr">
@@ -6817,11 +6817,11 @@
         </is>
       </c>
       <c r="P13" s="21" t="n">
-        <v>0</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="Q13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="R13" s="18" t="inlineStr">
@@ -6836,17 +6836,17 @@
       </c>
       <c r="T13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>security-reviewer-g4-f11</t>
         </is>
       </c>
       <c r="U13" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T13:56:46.057Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(F04): record G4 security review (pass)
Independent Security-Reviewer pass: no secret leakage in heal
forensics/PR body (redacted-summary regression test holds), no
merge/approve capability anywhere in registry-client.ts, nightly
sweep (scripts/self-heal.mjs) structurally cannot open a PR, and
agent-submitted heal scripts are dry-run + schema-validated before
ever touching the manifest or registry. Local build (npm run build)
and full suite (108 tests) pass. Tracker: reviewer set, gate -> G5.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6059,7 +6059,7 @@
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="R6" s="18" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>codex-gate-review</t>
+          <t>claude-f04-g4-security-reviewer</t>
         </is>
       </c>
       <c r="U6" s="18" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="V6" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T13:04:41.588Z</t>
+          <t>2026-07-17T14:00:32.944Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate tracker after F06 merge
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -5835,7 +5835,7 @@
         </is>
       </c>
       <c r="P4" s="21" t="n">
-        <v>0.9090909090909091</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
@@ -5994,72 +5994,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O6" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O6" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P6" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R6" s="18" t="inlineStr">
@@ -6069,22 +6069,22 @@
       </c>
       <c r="S6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex</t>
         </is>
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>claude-f04-g4-security-reviewer</t>
         </is>
       </c>
       <c r="U6" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V6" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T14:04:18.000Z</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="P7" s="21" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
@@ -6259,9 +6259,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="M8" s="23" t="inlineStr">
-        <is>
-          <t>In-Review</t>
+      <c r="M8" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="N8" s="19" t="inlineStr">
@@ -6269,17 +6269,17 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="O8" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O8" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P8" s="21" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="18" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R8" s="18" t="inlineStr">
@@ -6289,22 +6289,22 @@
       </c>
       <c r="S8" s="18" t="inlineStr">
         <is>
-          <t>codex-f06-builder</t>
+          <t>codex-f06-builder-repair</t>
         </is>
       </c>
       <c r="T8" s="18" t="inlineStr">
         <is>
-          <t>codex-f06-reviewer</t>
+          <t>security-reviewer-g4</t>
         </is>
       </c>
       <c r="U8" s="18" t="inlineStr">
         <is>
-          <t>In-Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V8" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T13:03:17.132Z</t>
+          <t>2026-07-17T14:11:00.000Z</t>
         </is>
       </c>
     </row>
@@ -6324,72 +6324,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O9" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O9" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P9" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R9" s="18" t="inlineStr">
@@ -6404,17 +6404,17 @@
       </c>
       <c r="T9" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex-f07-gate-reviewer</t>
         </is>
       </c>
       <c r="U9" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V9" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T13:14:10.819Z</t>
         </is>
       </c>
     </row>
@@ -6434,14 +6434,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr">
@@ -6449,57 +6449,57 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O10" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O10" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P10" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R10" s="18" t="inlineStr">
@@ -6514,17 +6514,17 @@
       </c>
       <c r="T10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Codex_F08_gate_reviewer</t>
         </is>
       </c>
       <c r="U10" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T12:52:18.246Z</t>
         </is>
       </c>
     </row>
@@ -6764,72 +6764,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K13" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N13" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O13" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O13" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P13" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R13" s="18" t="inlineStr">
@@ -6839,22 +6839,22 @@
       </c>
       <c r="S13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="T13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>security-reviewer-g4-f11; claude-batchA-g5-qa</t>
         </is>
       </c>
       <c r="U13" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V13" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T14:04:22.000Z</t>
         </is>
       </c>
     </row>
@@ -6874,9 +6874,9 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
@@ -6904,9 +6904,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
@@ -6935,11 +6935,11 @@
         </is>
       </c>
       <c r="P14" s="21" t="n">
-        <v>0</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="Q14" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="R14" s="18" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="U14" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Progress</t>
         </is>
       </c>
       <c r="V14" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T13:58:09.203Z</t>
         </is>
       </c>
     </row>
@@ -7754,44 +7754,44 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K22" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="L22" s="20" t="inlineStr">
@@ -7799,9 +7799,9 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="M22" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="M22" s="23" t="inlineStr">
+        <is>
+          <t>In-Review</t>
         </is>
       </c>
       <c r="N22" s="20" t="inlineStr">
@@ -7815,11 +7815,11 @@
         </is>
       </c>
       <c r="P22" s="21" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="Q22" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="R22" s="18" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="S22" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>builder-f20</t>
         </is>
       </c>
       <c r="T22" s="18" t="inlineStr">
@@ -7839,12 +7839,12 @@
       </c>
       <c r="U22" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>In-Prog</t>
         </is>
       </c>
       <c r="V22" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T19:30:00.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate tracker after F17 merge; lockfile sync
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6879,24 +6879,24 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I14" s="22" t="inlineStr">
@@ -6909,9 +6909,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="K14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="L14" s="20" t="inlineStr">
@@ -6919,27 +6919,27 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="M14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O14" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="M14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N14" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O14" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P14" s="21" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="Q14" s="18" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R14" s="18" t="inlineStr">
@@ -6949,22 +6949,22 @@
       </c>
       <c r="S14" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>codex-f12-builder</t>
         </is>
       </c>
       <c r="T14" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>claude-main-session-g2-g4-g5</t>
         </is>
       </c>
       <c r="U14" s="18" t="inlineStr">
         <is>
-          <t>In-Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V14" s="18" t="inlineStr">
         <is>
-          <t>2026-07-17T13:58:09.203Z</t>
+          <t>2026-07-17T14:10:00.000Z</t>
         </is>
       </c>
     </row>
@@ -7424,14 +7424,14 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="22" t="inlineStr">
@@ -7439,57 +7439,57 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="G19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I19" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="L19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="O19" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O19" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P19" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R19" s="18" t="inlineStr">
@@ -7499,22 +7499,22 @@
       </c>
       <c r="S19" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>engine-builder</t>
         </is>
       </c>
       <c r="T19" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G2-code-reviewer; claude-main-session-g6-reverify</t>
         </is>
       </c>
       <c r="U19" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V19" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T14:16:00.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate tracker after F13 merge
</commit_message>
<xml_diff>
--- a/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
+++ b/radical-pipeline/05-tracking/APImeMCP-Radical-Tracker.xlsx
@@ -6984,72 +6984,72 @@
           <t>Program 1</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="J15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="K15" s="22" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N15" s="22" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="M15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N15" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O15" s="20" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="O15" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="P15" s="21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="R15" s="18" t="inlineStr">
@@ -7059,22 +7059,22 @@
       </c>
       <c r="S15" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>engine-builder-f13</t>
         </is>
       </c>
       <c r="T15" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>code-reviewer-g2; claude-main-session-wiring-fix-and-g6</t>
         </is>
       </c>
       <c r="U15" s="18" t="inlineStr">
         <is>
-          <t>Not-started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="V15" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-17T14:28:00.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>